<commit_message>
feat : add and remove dokumen
</commit_message>
<xml_diff>
--- a/docs-v2/template/template_import_user.xlsx
+++ b/docs-v2/template/template_import_user.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\pacman\e-dashbord\docs-v2\template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\pacman\e-dashboard\docs-v2\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5CA203A6-2F92-4A64-835B-A2B75F7E1025}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{440BAD19-47BD-4F83-809D-0A3E7EE0EAAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2580" yWindow="2580" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="75" yWindow="1170" windowWidth="28725" windowHeight="10050" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="26">
   <si>
     <t>Template Import User Baru</t>
   </si>
@@ -86,6 +86,18 @@
   </si>
   <si>
     <t>PT MKO</t>
+  </si>
+  <si>
+    <t>admin</t>
+  </si>
+  <si>
+    <t>user</t>
+  </si>
+  <si>
+    <t>FAT Manager MKO</t>
+  </si>
+  <si>
+    <t>fat@mko.com</t>
   </si>
 </sst>
 </file>
@@ -130,9 +142,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -473,16 +486,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.796875" customWidth="1"/>
-    <col min="2" max="2" width="32.796875" customWidth="1"/>
-    <col min="3" max="3" width="48.796875" customWidth="1"/>
-    <col min="4" max="4" width="40.796875" customWidth="1"/>
+    <col min="1" max="1" width="24.75" customWidth="1"/>
+    <col min="2" max="2" width="32.75" customWidth="1"/>
+    <col min="3" max="3" width="48.75" customWidth="1"/>
+    <col min="4" max="4" width="40.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -490,7 +503,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="55.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" ht="55.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -504,7 +517,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -518,58 +531,87 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>10</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>13</v>
       </c>
+      <c r="C4" t="s">
+        <v>22</v>
+      </c>
       <c r="D4" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>11</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="C5" t="s">
+        <v>22</v>
+      </c>
       <c r="D5" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>12</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="C6" t="s">
+        <v>22</v>
+      </c>
       <c r="D6" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>16</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="C7" t="s">
+        <v>22</v>
+      </c>
       <c r="D7" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>17</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>19</v>
       </c>
+      <c r="C8" t="s">
+        <v>23</v>
+      </c>
       <c r="D8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" t="s">
         <v>21</v>
       </c>
     </row>
@@ -580,6 +622,7 @@
     <hyperlink ref="B6" r:id="rId3" xr:uid="{8F1F9A89-6D0E-4A03-BF1D-54D420B38267}"/>
     <hyperlink ref="B7" r:id="rId4" xr:uid="{0E05579D-8BBD-4869-92D9-35467754D281}"/>
     <hyperlink ref="B8" r:id="rId5" xr:uid="{D9AC99D9-95DD-4A17-B699-E9FA1FC4E8CF}"/>
+    <hyperlink ref="B9" r:id="rId6" xr:uid="{F7B21C14-31C0-4601-92B6-905831CE7EF4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>

</xml_diff>